<commit_message>
Support latest workbook and confirmed missing-month zero fill
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/consumption-latest.xlsx
+++ b/apps/web/public/templates/consumption-latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91983\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F178CF64-E060-4DE0-9388-4EB2E755CBEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801A14B9-5B7A-4AC0-83C5-96DFE301017E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="14235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="14595" windowHeight="21435" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Historic Consumption" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Drivers" sheetId="5" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Emissions!$C$1:$C$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Emissions!$C$1:$C$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Targets!$C$1:$C$73</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="55">
   <si>
     <t>Site Code</t>
   </si>
@@ -8891,7 +8891,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D1011"/>
+  <dimension ref="A1:D1012"/>
   <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="16.53125" customWidth="1"/>
@@ -9594,7 +9594,7 @@
         <v>2025</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D50" s="3">
         <v>0.4</v>
@@ -9608,10 +9608,10 @@
         <v>2025</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D51" s="3">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9622,10 +9622,10 @@
         <v>2025</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D52" s="3">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9636,10 +9636,10 @@
         <v>2025</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D53" s="3">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9650,10 +9650,10 @@
         <v>2025</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D54" s="3">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9664,10 +9664,10 @@
         <v>2025</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D55" s="3">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9678,10 +9678,10 @@
         <v>2025</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D56" s="3">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9692,10 +9692,10 @@
         <v>2025</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D57" s="3">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9706,10 +9706,10 @@
         <v>2025</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D58" s="3">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9720,10 +9720,10 @@
         <v>2025</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D59" s="3">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9734,10 +9734,10 @@
         <v>2025</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D60" s="3">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9745,13 +9745,13 @@
         <v>19</v>
       </c>
       <c r="B61" s="3">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D61" s="3">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9762,10 +9762,10 @@
         <v>2026</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D62" s="3">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9776,10 +9776,10 @@
         <v>2026</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D63" s="3">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9790,10 +9790,10 @@
         <v>2026</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D64" s="3">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9804,10 +9804,10 @@
         <v>2026</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D65" s="3">
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9818,10 +9818,10 @@
         <v>2026</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D66" s="3">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9832,10 +9832,10 @@
         <v>2026</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D67" s="3">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9846,10 +9846,10 @@
         <v>2026</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D68" s="3">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9860,10 +9860,10 @@
         <v>2026</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D69" s="3">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9874,10 +9874,10 @@
         <v>2026</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D70" s="3">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9888,10 +9888,10 @@
         <v>2026</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D71" s="3">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9902,24 +9902,24 @@
         <v>2026</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D72" s="3">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B73" s="3">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D73" s="3">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9930,10 +9930,10 @@
         <v>2025</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D74" s="3">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9944,10 +9944,10 @@
         <v>2025</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D75" s="3">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9958,10 +9958,10 @@
         <v>2025</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D76" s="3">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9972,10 +9972,10 @@
         <v>2025</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D77" s="3">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -9986,10 +9986,10 @@
         <v>2025</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D78" s="3">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10000,10 +10000,10 @@
         <v>2025</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D79" s="3">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="80" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10014,10 +10014,10 @@
         <v>2025</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D80" s="3">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10028,10 +10028,10 @@
         <v>2025</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D81" s="3">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10042,10 +10042,10 @@
         <v>2025</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D82" s="3">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10056,10 +10056,10 @@
         <v>2025</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D83" s="3">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10070,10 +10070,10 @@
         <v>2025</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D84" s="3">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10081,13 +10081,13 @@
         <v>11</v>
       </c>
       <c r="B85" s="3">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D85" s="3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10098,10 +10098,10 @@
         <v>2026</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D86" s="3">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10112,10 +10112,10 @@
         <v>2026</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D87" s="3">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10126,10 +10126,10 @@
         <v>2026</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D88" s="3">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10140,10 +10140,10 @@
         <v>2026</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D89" s="3">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10154,10 +10154,10 @@
         <v>2026</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D90" s="3">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10168,10 +10168,10 @@
         <v>2026</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D91" s="3">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10182,10 +10182,10 @@
         <v>2026</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D92" s="3">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10196,10 +10196,10 @@
         <v>2026</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D93" s="3">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10210,10 +10210,10 @@
         <v>2026</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D94" s="3">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10224,10 +10224,10 @@
         <v>2026</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D95" s="3">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -10238,17 +10238,25 @@
         <v>2026</v>
       </c>
       <c r="C96" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D96" s="3">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A97" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B97" s="3">
+        <v>2026</v>
+      </c>
+      <c r="C97" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D96" s="3">
+      <c r="D97" s="3">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A97" s="3"/>
-      <c r="B97" s="3"/>
-      <c r="C97" s="3"/>
-      <c r="D97" s="3"/>
     </row>
     <row r="98" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A98" s="3"/>
@@ -10316,7 +10324,12 @@
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
     </row>
-    <row r="109" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="109" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A109" s="3"/>
+      <c r="B109" s="3"/>
+      <c r="C109" s="3"/>
+      <c r="D109" s="3"/>
+    </row>
     <row r="110" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="111" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="112" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -11219,10 +11232,11 @@
     <row r="1009" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="1010" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="1011" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="1012" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
-  <autoFilter ref="C1:C108" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="C1:C109" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C108" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C109" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>